<commit_message>
Update Excel files for purchased and sold data
- Modified hd_purchased_hasCode.xlsx to reflect recent changes.
- Updated hd_purchased_initCode.xlsx with new entries.
- Revised hd_purchased_noCode.xlsx for accuracy.
- Adjusted hd_sold.xlsx to include the latest sales information.
</commit_message>
<xml_diff>
--- a/src/xlsx/hd_purchased_hasCode.xlsx
+++ b/src/xlsx/hd_purchased_hasCode.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/trungthanh.nguyen/Code/ScrappingData/src/xlsx/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{783FD4FD-72F0-1A41-BF53-5394669723A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CCEC31A-F0B2-C148-88D2-6B43562F434C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="970" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1334" uniqueCount="288">
   <si>
     <t>DANH SÁCH HÓA ĐƠN</t>
   </si>
@@ -698,6 +698,192 @@
   </si>
   <si>
     <t>4315</t>
+  </si>
+  <si>
+    <t>560758</t>
+  </si>
+  <si>
+    <t>04/07/2026</t>
+  </si>
+  <si>
+    <t>C26TMS</t>
+  </si>
+  <si>
+    <t>432205</t>
+  </si>
+  <si>
+    <t>13/07/2026</t>
+  </si>
+  <si>
+    <t>0101243150</t>
+  </si>
+  <si>
+    <t>Công ty cổ phần MISA</t>
+  </si>
+  <si>
+    <t>4725</t>
+  </si>
+  <si>
+    <t>14/07/2026</t>
+  </si>
+  <si>
+    <t>160614</t>
+  </si>
+  <si>
+    <t>01/07/2026</t>
+  </si>
+  <si>
+    <t>162135</t>
+  </si>
+  <si>
+    <t>02/07/2026</t>
+  </si>
+  <si>
+    <t>163731</t>
+  </si>
+  <si>
+    <t>03/07/2026</t>
+  </si>
+  <si>
+    <t>164574</t>
+  </si>
+  <si>
+    <t>166341</t>
+  </si>
+  <si>
+    <t>05/07/2026</t>
+  </si>
+  <si>
+    <t>171060</t>
+  </si>
+  <si>
+    <t>08/07/2026</t>
+  </si>
+  <si>
+    <t>173597</t>
+  </si>
+  <si>
+    <t>11/07/2026</t>
+  </si>
+  <si>
+    <t>174463</t>
+  </si>
+  <si>
+    <t>175649</t>
+  </si>
+  <si>
+    <t>12/07/2026</t>
+  </si>
+  <si>
+    <t>177266</t>
+  </si>
+  <si>
+    <t>179735</t>
+  </si>
+  <si>
+    <t>15/07/2026</t>
+  </si>
+  <si>
+    <t>179766</t>
+  </si>
+  <si>
+    <t>181679</t>
+  </si>
+  <si>
+    <t>16/07/2026</t>
+  </si>
+  <si>
+    <t>181681</t>
+  </si>
+  <si>
+    <t>185419</t>
+  </si>
+  <si>
+    <t>19/07/2026</t>
+  </si>
+  <si>
+    <t>186254</t>
+  </si>
+  <si>
+    <t>187908</t>
+  </si>
+  <si>
+    <t>20/07/2026</t>
+  </si>
+  <si>
+    <t>188776</t>
+  </si>
+  <si>
+    <t>21/07/2026</t>
+  </si>
+  <si>
+    <t>190824</t>
+  </si>
+  <si>
+    <t>22/07/2026</t>
+  </si>
+  <si>
+    <t>192737</t>
+  </si>
+  <si>
+    <t>24/07/2026</t>
+  </si>
+  <si>
+    <t>119</t>
+  </si>
+  <si>
+    <t>C26TAC</t>
+  </si>
+  <si>
+    <t>2389</t>
+  </si>
+  <si>
+    <t>06/07/2026</t>
+  </si>
+  <si>
+    <t>11407</t>
+  </si>
+  <si>
+    <t>25/07/2026</t>
+  </si>
+  <si>
+    <t>C26TYA</t>
+  </si>
+  <si>
+    <t>29252</t>
+  </si>
+  <si>
+    <t>17/07/2026</t>
+  </si>
+  <si>
+    <t>0318836678</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH ZALO PLATFORMS</t>
+  </si>
+  <si>
+    <t>Trung tâm Giáo dục nghề nghiệp Bách Việt</t>
+  </si>
+  <si>
+    <t>53 Nguyễn Đức Thuận, Phường Tân Bình, Tp. Hồ Chí Minh</t>
+  </si>
+  <si>
+    <t>C26THN</t>
+  </si>
+  <si>
+    <t>21</t>
+  </si>
+  <si>
+    <t>07/07/2026</t>
+  </si>
+  <si>
+    <t>0319381670</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH THƯƠNG MẠI &amp; DỊCH VỤ TỔNG HỢP 3HN</t>
+  </si>
+  <si>
+    <t>53 Nguyễn Đức Thuận, Phường Tân Bình, Thành phố Hồ Chí Minh</t>
   </si>
 </sst>
 </file>
@@ -811,18 +997,18 @@
     <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1158,7 +1344,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A3:S79"/>
+  <dimension ref="A3:S107"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7.83203125" customWidth="1"/>
@@ -1173,50 +1359,50 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A3" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="7"/>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
-      <c r="F3" s="7"/>
-      <c r="G3" s="7"/>
-      <c r="H3" s="7"/>
-      <c r="I3" s="7"/>
-      <c r="J3" s="7"/>
-      <c r="K3" s="7"/>
-      <c r="L3" s="7"/>
-      <c r="M3" s="7"/>
-      <c r="N3" s="7"/>
-      <c r="O3" s="7"/>
-      <c r="P3" s="7"/>
-      <c r="Q3" s="7"/>
-      <c r="R3" s="7"/>
-      <c r="S3" s="7"/>
+      <c r="A3" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="9"/>
+      <c r="I3" s="9"/>
+      <c r="J3" s="9"/>
+      <c r="K3" s="9"/>
+      <c r="L3" s="9"/>
+      <c r="M3" s="9"/>
+      <c r="N3" s="9"/>
+      <c r="O3" s="9"/>
+      <c r="P3" s="9"/>
+      <c r="Q3" s="9"/>
+      <c r="R3" s="9"/>
+      <c r="S3" s="9"/>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="7"/>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7"/>
-      <c r="I4" s="7"/>
-      <c r="J4" s="7"/>
-      <c r="K4" s="7"/>
-      <c r="L4" s="7"/>
-      <c r="M4" s="7"/>
-      <c r="N4" s="7"/>
-      <c r="O4" s="7"/>
-      <c r="P4" s="7"/>
-      <c r="Q4" s="7"/>
-      <c r="R4" s="7"/>
-      <c r="S4" s="7"/>
+      <c r="B4" s="9"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="9"/>
+      <c r="I4" s="9"/>
+      <c r="J4" s="9"/>
+      <c r="K4" s="9"/>
+      <c r="L4" s="9"/>
+      <c r="M4" s="9"/>
+      <c r="N4" s="9"/>
+      <c r="O4" s="9"/>
+      <c r="P4" s="9"/>
+      <c r="Q4" s="9"/>
+      <c r="R4" s="9"/>
+      <c r="S4" s="9"/>
     </row>
     <row r="6" spans="1:19" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
@@ -3371,7 +3557,7 @@
       <c r="B44" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C44" s="9" t="s">
+      <c r="C44" s="6" t="s">
         <v>34</v>
       </c>
       <c r="D44" s="2" t="s">
@@ -3383,29 +3569,29 @@
       <c r="F44" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="G44" s="9" t="s">
+      <c r="G44" s="6" t="s">
         <v>38</v>
       </c>
       <c r="H44" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="I44" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J44" s="9" t="s">
+      <c r="I44" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J44" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="K44" s="10">
+      <c r="K44" s="7">
         <v>150000</v>
       </c>
-      <c r="L44" s="10">
+      <c r="L44" s="7">
         <v>12000</v>
       </c>
-      <c r="M44" s="10">
-        <v>0</v>
-      </c>
-      <c r="N44" s="10"/>
-      <c r="O44" s="10">
+      <c r="M44" s="7">
+        <v>0</v>
+      </c>
+      <c r="N44" s="7"/>
+      <c r="O44" s="7">
         <v>162000</v>
       </c>
       <c r="P44" s="2" t="s">
@@ -3414,10 +3600,10 @@
       <c r="Q44" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="R44" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="S44" s="9" t="s">
+      <c r="R44" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S44" s="6" t="s">
         <v>33</v>
       </c>
     </row>
@@ -3428,7 +3614,7 @@
       <c r="B45" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C45" s="9" t="s">
+      <c r="C45" s="6" t="s">
         <v>34</v>
       </c>
       <c r="D45" s="2" t="s">
@@ -3440,29 +3626,29 @@
       <c r="F45" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="G45" s="9" t="s">
+      <c r="G45" s="6" t="s">
         <v>38</v>
       </c>
       <c r="H45" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="I45" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J45" s="9" t="s">
+      <c r="I45" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J45" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="K45" s="10">
+      <c r="K45" s="7">
         <v>30000000</v>
       </c>
-      <c r="L45" s="10">
-        <v>0</v>
-      </c>
-      <c r="M45" s="10">
-        <v>0</v>
-      </c>
-      <c r="N45" s="10"/>
-      <c r="O45" s="10">
+      <c r="L45" s="7">
+        <v>0</v>
+      </c>
+      <c r="M45" s="7">
+        <v>0</v>
+      </c>
+      <c r="N45" s="7"/>
+      <c r="O45" s="7">
         <v>30000000</v>
       </c>
       <c r="P45" s="2" t="s">
@@ -3471,10 +3657,10 @@
       <c r="Q45" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="R45" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="S45" s="9" t="s">
+      <c r="R45" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S45" s="6" t="s">
         <v>33</v>
       </c>
     </row>
@@ -3485,7 +3671,7 @@
       <c r="B46" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C46" s="9" t="s">
+      <c r="C46" s="6" t="s">
         <v>34</v>
       </c>
       <c r="D46" s="2" t="s">
@@ -3497,29 +3683,29 @@
       <c r="F46" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="G46" s="9" t="s">
+      <c r="G46" s="6" t="s">
         <v>38</v>
       </c>
       <c r="H46" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="I46" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J46" s="9" t="s">
+      <c r="I46" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J46" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="K46" s="10">
+      <c r="K46" s="7">
         <v>17400000</v>
       </c>
-      <c r="L46" s="10">
+      <c r="L46" s="7">
         <v>1200000</v>
       </c>
-      <c r="M46" s="10">
-        <v>0</v>
-      </c>
-      <c r="N46" s="10"/>
-      <c r="O46" s="10">
+      <c r="M46" s="7">
+        <v>0</v>
+      </c>
+      <c r="N46" s="7"/>
+      <c r="O46" s="7">
         <v>18600000</v>
       </c>
       <c r="P46" s="2" t="s">
@@ -3528,10 +3714,10 @@
       <c r="Q46" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="R46" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="S46" s="9" t="s">
+      <c r="R46" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S46" s="6" t="s">
         <v>33</v>
       </c>
     </row>
@@ -3542,7 +3728,7 @@
       <c r="B47" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C47" s="9" t="s">
+      <c r="C47" s="6" t="s">
         <v>154</v>
       </c>
       <c r="D47" s="2" t="s">
@@ -3554,29 +3740,29 @@
       <c r="F47" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="G47" s="9" t="s">
+      <c r="G47" s="6" t="s">
         <v>158</v>
       </c>
       <c r="H47" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="I47" s="9" t="s">
+      <c r="I47" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="J47" s="9" t="s">
+      <c r="J47" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="K47" s="10">
+      <c r="K47" s="7">
         <v>300000</v>
       </c>
-      <c r="L47" s="10">
+      <c r="L47" s="7">
         <v>24000</v>
       </c>
-      <c r="M47" s="10"/>
-      <c r="N47" s="10">
+      <c r="M47" s="7"/>
+      <c r="N47" s="7">
         <v>20000</v>
       </c>
-      <c r="O47" s="10">
+      <c r="O47" s="7">
         <v>344000</v>
       </c>
       <c r="P47" s="2" t="s">
@@ -3585,10 +3771,10 @@
       <c r="Q47" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="R47" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="S47" s="9" t="s">
+      <c r="R47" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S47" s="6" t="s">
         <v>33</v>
       </c>
     </row>
@@ -3599,7 +3785,7 @@
       <c r="B48" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C48" s="9" t="s">
+      <c r="C48" s="6" t="s">
         <v>47</v>
       </c>
       <c r="D48" s="2" t="s">
@@ -3611,29 +3797,29 @@
       <c r="F48" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="G48" s="9" t="s">
+      <c r="G48" s="6" t="s">
         <v>51</v>
       </c>
       <c r="H48" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="I48" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J48" s="9" t="s">
+      <c r="I48" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J48" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="K48" s="10">
+      <c r="K48" s="7">
         <v>700000</v>
       </c>
-      <c r="L48" s="10">
-        <v>0</v>
-      </c>
-      <c r="M48" s="10">
-        <v>0</v>
-      </c>
-      <c r="N48" s="10"/>
-      <c r="O48" s="10">
+      <c r="L48" s="7">
+        <v>0</v>
+      </c>
+      <c r="M48" s="7">
+        <v>0</v>
+      </c>
+      <c r="N48" s="7"/>
+      <c r="O48" s="7">
         <v>700000</v>
       </c>
       <c r="P48" s="2" t="s">
@@ -3642,10 +3828,10 @@
       <c r="Q48" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="R48" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="S48" s="9" t="s">
+      <c r="R48" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S48" s="6" t="s">
         <v>33</v>
       </c>
     </row>
@@ -3656,7 +3842,7 @@
       <c r="B49" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C49" s="9" t="s">
+      <c r="C49" s="6" t="s">
         <v>47</v>
       </c>
       <c r="D49" s="2" t="s">
@@ -3668,29 +3854,29 @@
       <c r="F49" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="G49" s="9" t="s">
+      <c r="G49" s="6" t="s">
         <v>51</v>
       </c>
       <c r="H49" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="I49" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J49" s="9" t="s">
+      <c r="I49" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J49" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="K49" s="10">
+      <c r="K49" s="7">
         <v>695000</v>
       </c>
-      <c r="L49" s="10">
-        <v>0</v>
-      </c>
-      <c r="M49" s="10">
-        <v>0</v>
-      </c>
-      <c r="N49" s="10"/>
-      <c r="O49" s="10">
+      <c r="L49" s="7">
+        <v>0</v>
+      </c>
+      <c r="M49" s="7">
+        <v>0</v>
+      </c>
+      <c r="N49" s="7"/>
+      <c r="O49" s="7">
         <v>695000</v>
       </c>
       <c r="P49" s="2" t="s">
@@ -3699,10 +3885,10 @@
       <c r="Q49" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="R49" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="S49" s="9" t="s">
+      <c r="R49" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S49" s="6" t="s">
         <v>33</v>
       </c>
     </row>
@@ -3713,7 +3899,7 @@
       <c r="B50" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C50" s="9" t="s">
+      <c r="C50" s="6" t="s">
         <v>47</v>
       </c>
       <c r="D50" s="2" t="s">
@@ -3725,29 +3911,29 @@
       <c r="F50" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="G50" s="9" t="s">
+      <c r="G50" s="6" t="s">
         <v>51</v>
       </c>
       <c r="H50" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="I50" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J50" s="9" t="s">
+      <c r="I50" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J50" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="K50" s="10">
+      <c r="K50" s="7">
         <v>530000</v>
       </c>
-      <c r="L50" s="10">
-        <v>0</v>
-      </c>
-      <c r="M50" s="10">
-        <v>0</v>
-      </c>
-      <c r="N50" s="10"/>
-      <c r="O50" s="10">
+      <c r="L50" s="7">
+        <v>0</v>
+      </c>
+      <c r="M50" s="7">
+        <v>0</v>
+      </c>
+      <c r="N50" s="7"/>
+      <c r="O50" s="7">
         <v>530000</v>
       </c>
       <c r="P50" s="2" t="s">
@@ -3756,10 +3942,10 @@
       <c r="Q50" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="R50" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="S50" s="9" t="s">
+      <c r="R50" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S50" s="6" t="s">
         <v>33</v>
       </c>
     </row>
@@ -3770,7 +3956,7 @@
       <c r="B51" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C51" s="9" t="s">
+      <c r="C51" s="6" t="s">
         <v>47</v>
       </c>
       <c r="D51" s="2" t="s">
@@ -3782,29 +3968,29 @@
       <c r="F51" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="G51" s="9" t="s">
+      <c r="G51" s="6" t="s">
         <v>51</v>
       </c>
       <c r="H51" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="I51" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J51" s="9" t="s">
+      <c r="I51" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J51" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="K51" s="10">
+      <c r="K51" s="7">
         <v>500000</v>
       </c>
-      <c r="L51" s="10">
-        <v>0</v>
-      </c>
-      <c r="M51" s="10">
-        <v>0</v>
-      </c>
-      <c r="N51" s="10"/>
-      <c r="O51" s="10">
+      <c r="L51" s="7">
+        <v>0</v>
+      </c>
+      <c r="M51" s="7">
+        <v>0</v>
+      </c>
+      <c r="N51" s="7"/>
+      <c r="O51" s="7">
         <v>500000</v>
       </c>
       <c r="P51" s="2" t="s">
@@ -3813,10 +3999,10 @@
       <c r="Q51" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="R51" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="S51" s="9" t="s">
+      <c r="R51" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S51" s="6" t="s">
         <v>33</v>
       </c>
     </row>
@@ -3827,7 +4013,7 @@
       <c r="B52" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C52" s="9" t="s">
+      <c r="C52" s="6" t="s">
         <v>47</v>
       </c>
       <c r="D52" s="2" t="s">
@@ -3839,29 +4025,29 @@
       <c r="F52" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="G52" s="9" t="s">
+      <c r="G52" s="6" t="s">
         <v>51</v>
       </c>
       <c r="H52" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="I52" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J52" s="9" t="s">
+      <c r="I52" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J52" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="K52" s="10">
+      <c r="K52" s="7">
         <v>700000</v>
       </c>
-      <c r="L52" s="10">
-        <v>0</v>
-      </c>
-      <c r="M52" s="10">
-        <v>0</v>
-      </c>
-      <c r="N52" s="10"/>
-      <c r="O52" s="10">
+      <c r="L52" s="7">
+        <v>0</v>
+      </c>
+      <c r="M52" s="7">
+        <v>0</v>
+      </c>
+      <c r="N52" s="7"/>
+      <c r="O52" s="7">
         <v>700000</v>
       </c>
       <c r="P52" s="2" t="s">
@@ -3870,10 +4056,10 @@
       <c r="Q52" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="R52" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="S52" s="9" t="s">
+      <c r="R52" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S52" s="6" t="s">
         <v>33</v>
       </c>
     </row>
@@ -3884,7 +4070,7 @@
       <c r="B53" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C53" s="9" t="s">
+      <c r="C53" s="6" t="s">
         <v>47</v>
       </c>
       <c r="D53" s="2" t="s">
@@ -3896,29 +4082,29 @@
       <c r="F53" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="G53" s="9" t="s">
+      <c r="G53" s="6" t="s">
         <v>51</v>
       </c>
       <c r="H53" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="I53" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J53" s="9" t="s">
+      <c r="I53" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J53" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="K53" s="10">
+      <c r="K53" s="7">
         <v>750000</v>
       </c>
-      <c r="L53" s="10">
-        <v>0</v>
-      </c>
-      <c r="M53" s="10">
-        <v>0</v>
-      </c>
-      <c r="N53" s="10"/>
-      <c r="O53" s="10">
+      <c r="L53" s="7">
+        <v>0</v>
+      </c>
+      <c r="M53" s="7">
+        <v>0</v>
+      </c>
+      <c r="N53" s="7"/>
+      <c r="O53" s="7">
         <v>750000</v>
       </c>
       <c r="P53" s="2" t="s">
@@ -3927,10 +4113,10 @@
       <c r="Q53" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="R53" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="S53" s="9" t="s">
+      <c r="R53" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S53" s="6" t="s">
         <v>33</v>
       </c>
     </row>
@@ -3941,7 +4127,7 @@
       <c r="B54" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C54" s="9" t="s">
+      <c r="C54" s="6" t="s">
         <v>47</v>
       </c>
       <c r="D54" s="2" t="s">
@@ -3953,29 +4139,29 @@
       <c r="F54" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="G54" s="9" t="s">
+      <c r="G54" s="6" t="s">
         <v>51</v>
       </c>
       <c r="H54" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="I54" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J54" s="9" t="s">
+      <c r="I54" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J54" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="K54" s="10">
+      <c r="K54" s="7">
         <v>500000</v>
       </c>
-      <c r="L54" s="10">
-        <v>0</v>
-      </c>
-      <c r="M54" s="10">
-        <v>0</v>
-      </c>
-      <c r="N54" s="10"/>
-      <c r="O54" s="10">
+      <c r="L54" s="7">
+        <v>0</v>
+      </c>
+      <c r="M54" s="7">
+        <v>0</v>
+      </c>
+      <c r="N54" s="7"/>
+      <c r="O54" s="7">
         <v>500000</v>
       </c>
       <c r="P54" s="2" t="s">
@@ -3984,10 +4170,10 @@
       <c r="Q54" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="R54" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="S54" s="9" t="s">
+      <c r="R54" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S54" s="6" t="s">
         <v>33</v>
       </c>
     </row>
@@ -3998,7 +4184,7 @@
       <c r="B55" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C55" s="9" t="s">
+      <c r="C55" s="6" t="s">
         <v>47</v>
       </c>
       <c r="D55" s="2" t="s">
@@ -4010,29 +4196,29 @@
       <c r="F55" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="G55" s="9" t="s">
+      <c r="G55" s="6" t="s">
         <v>51</v>
       </c>
       <c r="H55" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="I55" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J55" s="9" t="s">
+      <c r="I55" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J55" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="K55" s="10">
+      <c r="K55" s="7">
         <v>726068</v>
       </c>
-      <c r="L55" s="10">
-        <v>0</v>
-      </c>
-      <c r="M55" s="10">
-        <v>0</v>
-      </c>
-      <c r="N55" s="10"/>
-      <c r="O55" s="10">
+      <c r="L55" s="7">
+        <v>0</v>
+      </c>
+      <c r="M55" s="7">
+        <v>0</v>
+      </c>
+      <c r="N55" s="7"/>
+      <c r="O55" s="7">
         <v>726068</v>
       </c>
       <c r="P55" s="2" t="s">
@@ -4041,10 +4227,10 @@
       <c r="Q55" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="R55" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="S55" s="9" t="s">
+      <c r="R55" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S55" s="6" t="s">
         <v>33</v>
       </c>
     </row>
@@ -4055,7 +4241,7 @@
       <c r="B56" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C56" s="9" t="s">
+      <c r="C56" s="6" t="s">
         <v>47</v>
       </c>
       <c r="D56" s="2" t="s">
@@ -4067,29 +4253,29 @@
       <c r="F56" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="G56" s="9" t="s">
+      <c r="G56" s="6" t="s">
         <v>51</v>
       </c>
       <c r="H56" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="I56" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J56" s="9" t="s">
+      <c r="I56" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J56" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="K56" s="10">
+      <c r="K56" s="7">
         <v>500000</v>
       </c>
-      <c r="L56" s="10">
-        <v>0</v>
-      </c>
-      <c r="M56" s="10">
-        <v>0</v>
-      </c>
-      <c r="N56" s="10"/>
-      <c r="O56" s="10">
+      <c r="L56" s="7">
+        <v>0</v>
+      </c>
+      <c r="M56" s="7">
+        <v>0</v>
+      </c>
+      <c r="N56" s="7"/>
+      <c r="O56" s="7">
         <v>500000</v>
       </c>
       <c r="P56" s="2" t="s">
@@ -4098,10 +4284,10 @@
       <c r="Q56" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="R56" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="S56" s="9" t="s">
+      <c r="R56" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S56" s="6" t="s">
         <v>33</v>
       </c>
     </row>
@@ -4112,7 +4298,7 @@
       <c r="B57" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C57" s="9" t="s">
+      <c r="C57" s="6" t="s">
         <v>47</v>
       </c>
       <c r="D57" s="2" t="s">
@@ -4124,29 +4310,29 @@
       <c r="F57" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="G57" s="9" t="s">
+      <c r="G57" s="6" t="s">
         <v>51</v>
       </c>
       <c r="H57" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="I57" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J57" s="9" t="s">
+      <c r="I57" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J57" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="K57" s="10">
+      <c r="K57" s="7">
         <v>500000</v>
       </c>
-      <c r="L57" s="10">
-        <v>0</v>
-      </c>
-      <c r="M57" s="10">
-        <v>0</v>
-      </c>
-      <c r="N57" s="10"/>
-      <c r="O57" s="10">
+      <c r="L57" s="7">
+        <v>0</v>
+      </c>
+      <c r="M57" s="7">
+        <v>0</v>
+      </c>
+      <c r="N57" s="7"/>
+      <c r="O57" s="7">
         <v>500000</v>
       </c>
       <c r="P57" s="2" t="s">
@@ -4155,10 +4341,10 @@
       <c r="Q57" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="R57" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="S57" s="9" t="s">
+      <c r="R57" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S57" s="6" t="s">
         <v>33</v>
       </c>
     </row>
@@ -4169,7 +4355,7 @@
       <c r="B58" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C58" s="9" t="s">
+      <c r="C58" s="6" t="s">
         <v>47</v>
       </c>
       <c r="D58" s="2" t="s">
@@ -4181,29 +4367,29 @@
       <c r="F58" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="G58" s="9" t="s">
+      <c r="G58" s="6" t="s">
         <v>51</v>
       </c>
       <c r="H58" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="I58" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J58" s="9" t="s">
+      <c r="I58" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J58" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="K58" s="10">
+      <c r="K58" s="7">
         <v>700000</v>
       </c>
-      <c r="L58" s="10">
-        <v>0</v>
-      </c>
-      <c r="M58" s="10">
-        <v>0</v>
-      </c>
-      <c r="N58" s="10"/>
-      <c r="O58" s="10">
+      <c r="L58" s="7">
+        <v>0</v>
+      </c>
+      <c r="M58" s="7">
+        <v>0</v>
+      </c>
+      <c r="N58" s="7"/>
+      <c r="O58" s="7">
         <v>700000</v>
       </c>
       <c r="P58" s="2" t="s">
@@ -4212,10 +4398,10 @@
       <c r="Q58" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="R58" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="S58" s="9" t="s">
+      <c r="R58" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S58" s="6" t="s">
         <v>33</v>
       </c>
     </row>
@@ -4226,7 +4412,7 @@
       <c r="B59" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C59" s="9" t="s">
+      <c r="C59" s="6" t="s">
         <v>47</v>
       </c>
       <c r="D59" s="2" t="s">
@@ -4238,29 +4424,29 @@
       <c r="F59" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="G59" s="9" t="s">
+      <c r="G59" s="6" t="s">
         <v>51</v>
       </c>
       <c r="H59" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="I59" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J59" s="9" t="s">
+      <c r="I59" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J59" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="K59" s="10">
+      <c r="K59" s="7">
         <v>770044</v>
       </c>
-      <c r="L59" s="10">
-        <v>0</v>
-      </c>
-      <c r="M59" s="10">
-        <v>0</v>
-      </c>
-      <c r="N59" s="10"/>
-      <c r="O59" s="10">
+      <c r="L59" s="7">
+        <v>0</v>
+      </c>
+      <c r="M59" s="7">
+        <v>0</v>
+      </c>
+      <c r="N59" s="7"/>
+      <c r="O59" s="7">
         <v>770044</v>
       </c>
       <c r="P59" s="2" t="s">
@@ -4269,10 +4455,10 @@
       <c r="Q59" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="R59" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="S59" s="9" t="s">
+      <c r="R59" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S59" s="6" t="s">
         <v>33</v>
       </c>
     </row>
@@ -4283,7 +4469,7 @@
       <c r="B60" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C60" s="9" t="s">
+      <c r="C60" s="6" t="s">
         <v>47</v>
       </c>
       <c r="D60" s="2" t="s">
@@ -4295,29 +4481,29 @@
       <c r="F60" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="G60" s="9" t="s">
+      <c r="G60" s="6" t="s">
         <v>51</v>
       </c>
       <c r="H60" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="I60" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J60" s="9" t="s">
+      <c r="I60" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J60" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="K60" s="10">
+      <c r="K60" s="7">
         <v>700000</v>
       </c>
-      <c r="L60" s="10">
-        <v>0</v>
-      </c>
-      <c r="M60" s="10">
-        <v>0</v>
-      </c>
-      <c r="N60" s="10"/>
-      <c r="O60" s="10">
+      <c r="L60" s="7">
+        <v>0</v>
+      </c>
+      <c r="M60" s="7">
+        <v>0</v>
+      </c>
+      <c r="N60" s="7"/>
+      <c r="O60" s="7">
         <v>700000</v>
       </c>
       <c r="P60" s="2" t="s">
@@ -4326,10 +4512,10 @@
       <c r="Q60" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="R60" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="S60" s="9" t="s">
+      <c r="R60" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S60" s="6" t="s">
         <v>33</v>
       </c>
     </row>
@@ -4340,7 +4526,7 @@
       <c r="B61" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C61" s="9" t="s">
+      <c r="C61" s="6" t="s">
         <v>47</v>
       </c>
       <c r="D61" s="2" t="s">
@@ -4352,29 +4538,29 @@
       <c r="F61" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="G61" s="9" t="s">
+      <c r="G61" s="6" t="s">
         <v>51</v>
       </c>
       <c r="H61" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="I61" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J61" s="9" t="s">
+      <c r="I61" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J61" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="K61" s="10">
+      <c r="K61" s="7">
         <v>450000</v>
       </c>
-      <c r="L61" s="10">
-        <v>0</v>
-      </c>
-      <c r="M61" s="10">
-        <v>0</v>
-      </c>
-      <c r="N61" s="10"/>
-      <c r="O61" s="10">
+      <c r="L61" s="7">
+        <v>0</v>
+      </c>
+      <c r="M61" s="7">
+        <v>0</v>
+      </c>
+      <c r="N61" s="7"/>
+      <c r="O61" s="7">
         <v>450000</v>
       </c>
       <c r="P61" s="2" t="s">
@@ -4383,10 +4569,10 @@
       <c r="Q61" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="R61" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="S61" s="9" t="s">
+      <c r="R61" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S61" s="6" t="s">
         <v>33</v>
       </c>
     </row>
@@ -4397,7 +4583,7 @@
       <c r="B62" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C62" s="9" t="s">
+      <c r="C62" s="6" t="s">
         <v>47</v>
       </c>
       <c r="D62" s="2" t="s">
@@ -4409,29 +4595,29 @@
       <c r="F62" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="G62" s="9" t="s">
+      <c r="G62" s="6" t="s">
         <v>51</v>
       </c>
       <c r="H62" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="I62" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J62" s="9" t="s">
+      <c r="I62" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J62" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="K62" s="10">
+      <c r="K62" s="7">
         <v>546918</v>
       </c>
-      <c r="L62" s="10">
-        <v>0</v>
-      </c>
-      <c r="M62" s="10">
-        <v>0</v>
-      </c>
-      <c r="N62" s="10"/>
-      <c r="O62" s="10">
+      <c r="L62" s="7">
+        <v>0</v>
+      </c>
+      <c r="M62" s="7">
+        <v>0</v>
+      </c>
+      <c r="N62" s="7"/>
+      <c r="O62" s="7">
         <v>546918</v>
       </c>
       <c r="P62" s="2" t="s">
@@ -4440,10 +4626,10 @@
       <c r="Q62" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="R62" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="S62" s="9" t="s">
+      <c r="R62" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S62" s="6" t="s">
         <v>33</v>
       </c>
     </row>
@@ -4454,7 +4640,7 @@
       <c r="B63" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C63" s="9" t="s">
+      <c r="C63" s="6" t="s">
         <v>47</v>
       </c>
       <c r="D63" s="2" t="s">
@@ -4466,29 +4652,29 @@
       <c r="F63" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="G63" s="9" t="s">
+      <c r="G63" s="6" t="s">
         <v>51</v>
       </c>
       <c r="H63" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="I63" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J63" s="9" t="s">
+      <c r="I63" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J63" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="K63" s="10">
+      <c r="K63" s="7">
         <v>800000</v>
       </c>
-      <c r="L63" s="10">
-        <v>0</v>
-      </c>
-      <c r="M63" s="10">
-        <v>0</v>
-      </c>
-      <c r="N63" s="10"/>
-      <c r="O63" s="10">
+      <c r="L63" s="7">
+        <v>0</v>
+      </c>
+      <c r="M63" s="7">
+        <v>0</v>
+      </c>
+      <c r="N63" s="7"/>
+      <c r="O63" s="7">
         <v>800000</v>
       </c>
       <c r="P63" s="2" t="s">
@@ -4497,10 +4683,10 @@
       <c r="Q63" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="R63" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="S63" s="9" t="s">
+      <c r="R63" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S63" s="6" t="s">
         <v>33</v>
       </c>
     </row>
@@ -4511,7 +4697,7 @@
       <c r="B64" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C64" s="9" t="s">
+      <c r="C64" s="6" t="s">
         <v>47</v>
       </c>
       <c r="D64" s="2" t="s">
@@ -4523,29 +4709,29 @@
       <c r="F64" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="G64" s="9" t="s">
+      <c r="G64" s="6" t="s">
         <v>51</v>
       </c>
       <c r="H64" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="I64" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J64" s="9" t="s">
+      <c r="I64" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J64" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="K64" s="10">
+      <c r="K64" s="7">
         <v>500000</v>
       </c>
-      <c r="L64" s="10">
-        <v>0</v>
-      </c>
-      <c r="M64" s="10">
-        <v>0</v>
-      </c>
-      <c r="N64" s="10"/>
-      <c r="O64" s="10">
+      <c r="L64" s="7">
+        <v>0</v>
+      </c>
+      <c r="M64" s="7">
+        <v>0</v>
+      </c>
+      <c r="N64" s="7"/>
+      <c r="O64" s="7">
         <v>500000</v>
       </c>
       <c r="P64" s="2" t="s">
@@ -4554,10 +4740,10 @@
       <c r="Q64" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="R64" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="S64" s="9" t="s">
+      <c r="R64" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S64" s="6" t="s">
         <v>33</v>
       </c>
     </row>
@@ -4568,7 +4754,7 @@
       <c r="B65" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C65" s="9" t="s">
+      <c r="C65" s="6" t="s">
         <v>47</v>
       </c>
       <c r="D65" s="2" t="s">
@@ -4580,29 +4766,29 @@
       <c r="F65" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="G65" s="9" t="s">
+      <c r="G65" s="6" t="s">
         <v>51</v>
       </c>
       <c r="H65" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="I65" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J65" s="9" t="s">
+      <c r="I65" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J65" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="K65" s="10">
+      <c r="K65" s="7">
         <v>677522</v>
       </c>
-      <c r="L65" s="10">
-        <v>0</v>
-      </c>
-      <c r="M65" s="10">
-        <v>0</v>
-      </c>
-      <c r="N65" s="10"/>
-      <c r="O65" s="10">
+      <c r="L65" s="7">
+        <v>0</v>
+      </c>
+      <c r="M65" s="7">
+        <v>0</v>
+      </c>
+      <c r="N65" s="7"/>
+      <c r="O65" s="7">
         <v>677522</v>
       </c>
       <c r="P65" s="2" t="s">
@@ -4611,10 +4797,10 @@
       <c r="Q65" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="R65" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="S65" s="9" t="s">
+      <c r="R65" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S65" s="6" t="s">
         <v>33</v>
       </c>
     </row>
@@ -4625,7 +4811,7 @@
       <c r="B66" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C66" s="9" t="s">
+      <c r="C66" s="6" t="s">
         <v>47</v>
       </c>
       <c r="D66" s="2" t="s">
@@ -4637,29 +4823,29 @@
       <c r="F66" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="G66" s="9" t="s">
+      <c r="G66" s="6" t="s">
         <v>51</v>
       </c>
       <c r="H66" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="I66" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J66" s="9" t="s">
+      <c r="I66" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J66" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="K66" s="10">
+      <c r="K66" s="7">
         <v>700000</v>
       </c>
-      <c r="L66" s="10">
-        <v>0</v>
-      </c>
-      <c r="M66" s="10">
-        <v>0</v>
-      </c>
-      <c r="N66" s="10"/>
-      <c r="O66" s="10">
+      <c r="L66" s="7">
+        <v>0</v>
+      </c>
+      <c r="M66" s="7">
+        <v>0</v>
+      </c>
+      <c r="N66" s="7"/>
+      <c r="O66" s="7">
         <v>700000</v>
       </c>
       <c r="P66" s="2" t="s">
@@ -4668,10 +4854,10 @@
       <c r="Q66" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="R66" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="S66" s="9" t="s">
+      <c r="R66" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S66" s="6" t="s">
         <v>33</v>
       </c>
     </row>
@@ -4682,7 +4868,7 @@
       <c r="B67" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C67" s="9" t="s">
+      <c r="C67" s="6" t="s">
         <v>47</v>
       </c>
       <c r="D67" s="2" t="s">
@@ -4694,29 +4880,29 @@
       <c r="F67" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="G67" s="9" t="s">
+      <c r="G67" s="6" t="s">
         <v>51</v>
       </c>
       <c r="H67" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="I67" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J67" s="9" t="s">
+      <c r="I67" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J67" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="K67" s="10">
+      <c r="K67" s="7">
         <v>456000</v>
       </c>
-      <c r="L67" s="10">
-        <v>0</v>
-      </c>
-      <c r="M67" s="10">
-        <v>0</v>
-      </c>
-      <c r="N67" s="10"/>
-      <c r="O67" s="10">
+      <c r="L67" s="7">
+        <v>0</v>
+      </c>
+      <c r="M67" s="7">
+        <v>0</v>
+      </c>
+      <c r="N67" s="7"/>
+      <c r="O67" s="7">
         <v>456000</v>
       </c>
       <c r="P67" s="2" t="s">
@@ -4725,10 +4911,10 @@
       <c r="Q67" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="R67" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="S67" s="9" t="s">
+      <c r="R67" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S67" s="6" t="s">
         <v>33</v>
       </c>
     </row>
@@ -4739,7 +4925,7 @@
       <c r="B68" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C68" s="9" t="s">
+      <c r="C68" s="6" t="s">
         <v>47</v>
       </c>
       <c r="D68" s="2" t="s">
@@ -4751,29 +4937,29 @@
       <c r="F68" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="G68" s="9" t="s">
+      <c r="G68" s="6" t="s">
         <v>51</v>
       </c>
       <c r="H68" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="I68" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J68" s="9" t="s">
+      <c r="I68" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J68" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="K68" s="10">
+      <c r="K68" s="7">
         <v>700000</v>
       </c>
-      <c r="L68" s="10">
-        <v>0</v>
-      </c>
-      <c r="M68" s="10">
-        <v>0</v>
-      </c>
-      <c r="N68" s="10"/>
-      <c r="O68" s="10">
+      <c r="L68" s="7">
+        <v>0</v>
+      </c>
+      <c r="M68" s="7">
+        <v>0</v>
+      </c>
+      <c r="N68" s="7"/>
+      <c r="O68" s="7">
         <v>700000</v>
       </c>
       <c r="P68" s="2" t="s">
@@ -4782,10 +4968,10 @@
       <c r="Q68" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="R68" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="S68" s="9" t="s">
+      <c r="R68" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S68" s="6" t="s">
         <v>33</v>
       </c>
     </row>
@@ -4796,7 +4982,7 @@
       <c r="B69" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C69" s="9" t="s">
+      <c r="C69" s="6" t="s">
         <v>47</v>
       </c>
       <c r="D69" s="2" t="s">
@@ -4808,29 +4994,29 @@
       <c r="F69" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="G69" s="9" t="s">
+      <c r="G69" s="6" t="s">
         <v>51</v>
       </c>
       <c r="H69" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="I69" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J69" s="9" t="s">
+      <c r="I69" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J69" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="K69" s="10">
+      <c r="K69" s="7">
         <v>480000</v>
       </c>
-      <c r="L69" s="10">
-        <v>0</v>
-      </c>
-      <c r="M69" s="10">
-        <v>0</v>
-      </c>
-      <c r="N69" s="10"/>
-      <c r="O69" s="10">
+      <c r="L69" s="7">
+        <v>0</v>
+      </c>
+      <c r="M69" s="7">
+        <v>0</v>
+      </c>
+      <c r="N69" s="7"/>
+      <c r="O69" s="7">
         <v>480000</v>
       </c>
       <c r="P69" s="2" t="s">
@@ -4839,10 +5025,10 @@
       <c r="Q69" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="R69" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="S69" s="9" t="s">
+      <c r="R69" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S69" s="6" t="s">
         <v>33</v>
       </c>
     </row>
@@ -4853,7 +5039,7 @@
       <c r="B70" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C70" s="9" t="s">
+      <c r="C70" s="6" t="s">
         <v>47</v>
       </c>
       <c r="D70" s="2" t="s">
@@ -4865,29 +5051,29 @@
       <c r="F70" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="G70" s="9" t="s">
+      <c r="G70" s="6" t="s">
         <v>51</v>
       </c>
       <c r="H70" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="I70" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J70" s="9" t="s">
+      <c r="I70" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J70" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="K70" s="10">
+      <c r="K70" s="7">
         <v>500000</v>
       </c>
-      <c r="L70" s="10">
-        <v>0</v>
-      </c>
-      <c r="M70" s="10">
-        <v>0</v>
-      </c>
-      <c r="N70" s="10"/>
-      <c r="O70" s="10">
+      <c r="L70" s="7">
+        <v>0</v>
+      </c>
+      <c r="M70" s="7">
+        <v>0</v>
+      </c>
+      <c r="N70" s="7"/>
+      <c r="O70" s="7">
         <v>500000</v>
       </c>
       <c r="P70" s="2" t="s">
@@ -4896,10 +5082,10 @@
       <c r="Q70" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="R70" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="S70" s="9" t="s">
+      <c r="R70" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S70" s="6" t="s">
         <v>33</v>
       </c>
     </row>
@@ -4910,7 +5096,7 @@
       <c r="B71" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C71" s="9" t="s">
+      <c r="C71" s="6" t="s">
         <v>197</v>
       </c>
       <c r="D71" s="2" t="s">
@@ -4922,29 +5108,29 @@
       <c r="F71" s="2" t="s">
         <v>199</v>
       </c>
-      <c r="G71" s="9" t="s">
+      <c r="G71" s="6" t="s">
         <v>200</v>
       </c>
       <c r="H71" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="I71" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J71" s="9" t="s">
+      <c r="I71" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J71" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="K71" s="10">
+      <c r="K71" s="7">
         <v>1032800</v>
       </c>
-      <c r="L71" s="10">
+      <c r="L71" s="7">
         <v>95280</v>
       </c>
-      <c r="M71" s="10">
-        <v>0</v>
-      </c>
-      <c r="N71" s="10"/>
-      <c r="O71" s="10">
+      <c r="M71" s="7">
+        <v>0</v>
+      </c>
+      <c r="N71" s="7"/>
+      <c r="O71" s="7">
         <v>1128080</v>
       </c>
       <c r="P71" s="2" t="s">
@@ -4953,10 +5139,10 @@
       <c r="Q71" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="R71" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="S71" s="9" t="s">
+      <c r="R71" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S71" s="6" t="s">
         <v>33</v>
       </c>
     </row>
@@ -4967,7 +5153,7 @@
       <c r="B72" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C72" s="9" t="s">
+      <c r="C72" s="6" t="s">
         <v>100</v>
       </c>
       <c r="D72" s="2" t="s">
@@ -4979,29 +5165,29 @@
       <c r="F72" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="G72" s="9" t="s">
+      <c r="G72" s="6" t="s">
         <v>103</v>
       </c>
       <c r="H72" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="I72" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J72" s="9" t="s">
+      <c r="I72" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J72" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="K72" s="10">
+      <c r="K72" s="7">
         <v>159509260</v>
       </c>
-      <c r="L72" s="10">
+      <c r="L72" s="7">
         <v>12760740</v>
       </c>
-      <c r="M72" s="10">
-        <v>0</v>
-      </c>
-      <c r="N72" s="10"/>
-      <c r="O72" s="10">
+      <c r="M72" s="7">
+        <v>0</v>
+      </c>
+      <c r="N72" s="7"/>
+      <c r="O72" s="7">
         <v>172270000</v>
       </c>
       <c r="P72" s="2" t="s">
@@ -5010,10 +5196,10 @@
       <c r="Q72" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="R72" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="S72" s="9" t="s">
+      <c r="R72" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S72" s="6" t="s">
         <v>33</v>
       </c>
     </row>
@@ -5024,7 +5210,7 @@
       <c r="B73" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C73" s="9" t="s">
+      <c r="C73" s="6" t="s">
         <v>202</v>
       </c>
       <c r="D73" s="2" t="s">
@@ -5036,29 +5222,29 @@
       <c r="F73" s="2" t="s">
         <v>205</v>
       </c>
-      <c r="G73" s="9" t="s">
+      <c r="G73" s="6" t="s">
         <v>206</v>
       </c>
       <c r="H73" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="I73" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J73" s="9" t="s">
+      <c r="I73" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J73" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="K73" s="10">
+      <c r="K73" s="7">
         <v>10694445</v>
       </c>
-      <c r="L73" s="10">
+      <c r="L73" s="7">
         <v>855555</v>
       </c>
-      <c r="M73" s="10">
-        <v>0</v>
-      </c>
-      <c r="N73" s="10"/>
-      <c r="O73" s="10">
+      <c r="M73" s="7">
+        <v>0</v>
+      </c>
+      <c r="N73" s="7"/>
+      <c r="O73" s="7">
         <v>11550000</v>
       </c>
       <c r="P73" s="2" t="s">
@@ -5067,10 +5253,10 @@
       <c r="Q73" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="R73" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="S73" s="9" t="s">
+      <c r="R73" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S73" s="6" t="s">
         <v>33</v>
       </c>
     </row>
@@ -5081,7 +5267,7 @@
       <c r="B74" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C74" s="9" t="s">
+      <c r="C74" s="6" t="s">
         <v>207</v>
       </c>
       <c r="D74" s="2" t="s">
@@ -5093,29 +5279,29 @@
       <c r="F74" s="2" t="s">
         <v>209</v>
       </c>
-      <c r="G74" s="9" t="s">
+      <c r="G74" s="6" t="s">
         <v>210</v>
       </c>
       <c r="H74" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="I74" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J74" s="9" t="s">
+      <c r="I74" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J74" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="K74" s="10">
+      <c r="K74" s="7">
         <v>4450000</v>
       </c>
-      <c r="L74" s="10">
+      <c r="L74" s="7">
         <v>356000</v>
       </c>
-      <c r="M74" s="10">
-        <v>0</v>
-      </c>
-      <c r="N74" s="10"/>
-      <c r="O74" s="10">
+      <c r="M74" s="7">
+        <v>0</v>
+      </c>
+      <c r="N74" s="7"/>
+      <c r="O74" s="7">
         <v>4806000</v>
       </c>
       <c r="P74" s="2" t="s">
@@ -5124,10 +5310,10 @@
       <c r="Q74" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="R74" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="S74" s="9" t="s">
+      <c r="R74" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S74" s="6" t="s">
         <v>33</v>
       </c>
     </row>
@@ -5138,7 +5324,7 @@
       <c r="B75" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C75" s="9" t="s">
+      <c r="C75" s="6" t="s">
         <v>211</v>
       </c>
       <c r="D75" s="2" t="s">
@@ -5150,29 +5336,29 @@
       <c r="F75" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="G75" s="9" t="s">
+      <c r="G75" s="6" t="s">
         <v>214</v>
       </c>
       <c r="H75" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="I75" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J75" s="9" t="s">
+      <c r="I75" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J75" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="K75" s="10">
+      <c r="K75" s="7">
         <v>8880000</v>
       </c>
-      <c r="L75" s="10">
-        <v>0</v>
-      </c>
-      <c r="M75" s="10">
-        <v>0</v>
-      </c>
-      <c r="N75" s="10"/>
-      <c r="O75" s="10">
+      <c r="L75" s="7">
+        <v>0</v>
+      </c>
+      <c r="M75" s="7">
+        <v>0</v>
+      </c>
+      <c r="N75" s="7"/>
+      <c r="O75" s="7">
         <v>8880000</v>
       </c>
       <c r="P75" s="2" t="s">
@@ -5181,10 +5367,10 @@
       <c r="Q75" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="R75" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="S75" s="9" t="s">
+      <c r="R75" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S75" s="6" t="s">
         <v>33</v>
       </c>
     </row>
@@ -5195,7 +5381,7 @@
       <c r="B76" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C76" s="9" t="s">
+      <c r="C76" s="6" t="s">
         <v>215</v>
       </c>
       <c r="D76" s="2" t="s">
@@ -5207,29 +5393,29 @@
       <c r="F76" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="G76" s="9" t="s">
+      <c r="G76" s="6" t="s">
         <v>219</v>
       </c>
       <c r="H76" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="I76" s="9" t="s">
+      <c r="I76" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="J76" s="9" t="s">
+      <c r="J76" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="K76" s="10">
+      <c r="K76" s="7">
         <v>859964</v>
       </c>
-      <c r="L76" s="10">
-        <v>0</v>
-      </c>
-      <c r="M76" s="10">
-        <v>0</v>
-      </c>
-      <c r="N76" s="10"/>
-      <c r="O76" s="10">
+      <c r="L76" s="7">
+        <v>0</v>
+      </c>
+      <c r="M76" s="7">
+        <v>0</v>
+      </c>
+      <c r="N76" s="7"/>
+      <c r="O76" s="7">
         <v>859964</v>
       </c>
       <c r="P76" s="2" t="s">
@@ -5238,10 +5424,10 @@
       <c r="Q76" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="R76" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="S76" s="9" t="s">
+      <c r="R76" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S76" s="6" t="s">
         <v>33</v>
       </c>
     </row>
@@ -5252,7 +5438,7 @@
       <c r="B77" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C77" s="9" t="s">
+      <c r="C77" s="6" t="s">
         <v>220</v>
       </c>
       <c r="D77" s="2" t="s">
@@ -5264,29 +5450,29 @@
       <c r="F77" s="2" t="s">
         <v>222</v>
       </c>
-      <c r="G77" s="9" t="s">
+      <c r="G77" s="6" t="s">
         <v>223</v>
       </c>
       <c r="H77" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="I77" s="9" t="s">
+      <c r="I77" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="J77" s="9" t="s">
+      <c r="J77" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="K77" s="10">
+      <c r="K77" s="7">
         <v>700437</v>
       </c>
-      <c r="L77" s="10">
-        <v>0</v>
-      </c>
-      <c r="M77" s="10">
-        <v>0</v>
-      </c>
-      <c r="N77" s="10"/>
-      <c r="O77" s="10">
+      <c r="L77" s="7">
+        <v>0</v>
+      </c>
+      <c r="M77" s="7">
+        <v>0</v>
+      </c>
+      <c r="N77" s="7"/>
+      <c r="O77" s="7">
         <v>700437</v>
       </c>
       <c r="P77" s="2" t="s">
@@ -5295,10 +5481,10 @@
       <c r="Q77" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="R77" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="S77" s="9" t="s">
+      <c r="R77" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S77" s="6" t="s">
         <v>33</v>
       </c>
     </row>
@@ -5309,7 +5495,7 @@
       <c r="B78" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C78" s="9" t="s">
+      <c r="C78" s="6" t="s">
         <v>139</v>
       </c>
       <c r="D78" s="2" t="s">
@@ -5321,29 +5507,29 @@
       <c r="F78" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="G78" s="9" t="s">
+      <c r="G78" s="6" t="s">
         <v>142</v>
       </c>
       <c r="H78" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="I78" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J78" s="9" t="s">
+      <c r="I78" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J78" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="K78" s="10">
+      <c r="K78" s="7">
         <v>300000</v>
       </c>
-      <c r="L78" s="10">
+      <c r="L78" s="7">
         <v>24000</v>
       </c>
-      <c r="M78" s="10"/>
-      <c r="N78" s="10">
+      <c r="M78" s="7"/>
+      <c r="N78" s="7">
         <v>20000</v>
       </c>
-      <c r="O78" s="10">
+      <c r="O78" s="7">
         <v>344000</v>
       </c>
       <c r="P78" s="2" t="s">
@@ -5352,10 +5538,10 @@
       <c r="Q78" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="R78" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="S78" s="9" t="s">
+      <c r="R78" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S78" s="6" t="s">
         <v>33</v>
       </c>
     </row>
@@ -5366,7 +5552,7 @@
       <c r="B79" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C79" s="9" t="s">
+      <c r="C79" s="6" t="s">
         <v>77</v>
       </c>
       <c r="D79" s="2" t="s">
@@ -5378,27 +5564,27 @@
       <c r="F79" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="G79" s="9" t="s">
+      <c r="G79" s="6" t="s">
         <v>142</v>
       </c>
       <c r="H79" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="I79" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J79" s="9" t="s">
+      <c r="I79" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J79" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="K79" s="10">
+      <c r="K79" s="7">
         <v>300000</v>
       </c>
-      <c r="L79" s="10">
+      <c r="L79" s="7">
         <v>24000</v>
       </c>
-      <c r="M79" s="10"/>
-      <c r="N79" s="10"/>
-      <c r="O79" s="10">
+      <c r="M79" s="7"/>
+      <c r="N79" s="7"/>
+      <c r="O79" s="7">
         <v>324000</v>
       </c>
       <c r="P79" s="2" t="s">
@@ -5407,10 +5593,1600 @@
       <c r="Q79" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="R79" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="S79" s="9" t="s">
+      <c r="R79" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S79" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="80" spans="1:19" ht="46" x14ac:dyDescent="0.2">
+      <c r="A80" s="2">
+        <v>1</v>
+      </c>
+      <c r="B80" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C80" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D80" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="E80" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="F80" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="G80" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="H80" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I80" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J80" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="K80" s="7">
+        <v>850036</v>
+      </c>
+      <c r="L80" s="7">
+        <v>0</v>
+      </c>
+      <c r="M80" s="7">
+        <v>0</v>
+      </c>
+      <c r="N80" s="7"/>
+      <c r="O80" s="7">
+        <v>850036</v>
+      </c>
+      <c r="P80" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q80" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="R80" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S80" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="81" spans="1:19" ht="31" x14ac:dyDescent="0.2">
+      <c r="A81" s="2">
+        <v>2</v>
+      </c>
+      <c r="B81" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C81" s="6" t="s">
+        <v>228</v>
+      </c>
+      <c r="D81" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="E81" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="F81" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="G81" s="6" t="s">
+        <v>232</v>
+      </c>
+      <c r="H81" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I81" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="J81" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="K81" s="7">
+        <v>16950000</v>
+      </c>
+      <c r="L81" s="7">
+        <v>0</v>
+      </c>
+      <c r="M81" s="7">
+        <v>0</v>
+      </c>
+      <c r="N81" s="7"/>
+      <c r="O81" s="7">
+        <v>16950000</v>
+      </c>
+      <c r="P81" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q81" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="R81" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S81" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="82" spans="1:19" ht="46" x14ac:dyDescent="0.2">
+      <c r="A82" s="2">
+        <v>3</v>
+      </c>
+      <c r="B82" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C82" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D82" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="E82" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="F82" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="G82" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="H82" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I82" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J82" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="K82" s="7">
+        <v>8400000</v>
+      </c>
+      <c r="L82" s="7">
+        <v>0</v>
+      </c>
+      <c r="M82" s="7">
+        <v>0</v>
+      </c>
+      <c r="N82" s="7"/>
+      <c r="O82" s="7">
+        <v>8400000</v>
+      </c>
+      <c r="P82" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q82" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="R82" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S82" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="83" spans="1:19" ht="46" x14ac:dyDescent="0.2">
+      <c r="A83" s="2">
+        <v>4</v>
+      </c>
+      <c r="B83" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C83" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D83" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="E83" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="F83" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="G83" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="H83" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I83" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J83" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="K83" s="7">
+        <v>600000</v>
+      </c>
+      <c r="L83" s="7">
+        <v>0</v>
+      </c>
+      <c r="M83" s="7">
+        <v>0</v>
+      </c>
+      <c r="N83" s="7"/>
+      <c r="O83" s="7">
+        <v>600000</v>
+      </c>
+      <c r="P83" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q83" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="R83" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S83" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="84" spans="1:19" ht="46" x14ac:dyDescent="0.2">
+      <c r="A84" s="2">
+        <v>5</v>
+      </c>
+      <c r="B84" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C84" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D84" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="E84" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="F84" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="G84" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="H84" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I84" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J84" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="K84" s="7">
+        <v>400036</v>
+      </c>
+      <c r="L84" s="7">
+        <v>0</v>
+      </c>
+      <c r="M84" s="7">
+        <v>0</v>
+      </c>
+      <c r="N84" s="7"/>
+      <c r="O84" s="7">
+        <v>400036</v>
+      </c>
+      <c r="P84" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q84" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="R84" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S84" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="85" spans="1:19" ht="46" x14ac:dyDescent="0.2">
+      <c r="A85" s="2">
+        <v>6</v>
+      </c>
+      <c r="B85" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C85" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D85" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="E85" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="F85" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="G85" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="H85" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I85" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J85" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="K85" s="7">
+        <v>362338</v>
+      </c>
+      <c r="L85" s="7">
+        <v>0</v>
+      </c>
+      <c r="M85" s="7">
+        <v>0</v>
+      </c>
+      <c r="N85" s="7"/>
+      <c r="O85" s="7">
+        <v>362338</v>
+      </c>
+      <c r="P85" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q85" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="R85" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S85" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="86" spans="1:19" ht="46" x14ac:dyDescent="0.2">
+      <c r="A86" s="2">
+        <v>7</v>
+      </c>
+      <c r="B86" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C86" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D86" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="E86" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="F86" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="G86" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="H86" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I86" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J86" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="K86" s="7">
+        <v>450000</v>
+      </c>
+      <c r="L86" s="7">
+        <v>0</v>
+      </c>
+      <c r="M86" s="7">
+        <v>0</v>
+      </c>
+      <c r="N86" s="7"/>
+      <c r="O86" s="7">
+        <v>450000</v>
+      </c>
+      <c r="P86" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q86" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="R86" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S86" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="87" spans="1:19" ht="46" x14ac:dyDescent="0.2">
+      <c r="A87" s="2">
+        <v>8</v>
+      </c>
+      <c r="B87" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C87" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D87" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="E87" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="F87" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="G87" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="H87" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I87" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J87" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="K87" s="7">
+        <v>414731</v>
+      </c>
+      <c r="L87" s="7">
+        <v>0</v>
+      </c>
+      <c r="M87" s="7">
+        <v>0</v>
+      </c>
+      <c r="N87" s="7"/>
+      <c r="O87" s="7">
+        <v>414731</v>
+      </c>
+      <c r="P87" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q87" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="R87" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S87" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="88" spans="1:19" ht="46" x14ac:dyDescent="0.2">
+      <c r="A88" s="2">
+        <v>9</v>
+      </c>
+      <c r="B88" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C88" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D88" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="E88" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="F88" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="G88" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="H88" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I88" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J88" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="K88" s="7">
+        <v>501555</v>
+      </c>
+      <c r="L88" s="7">
+        <v>0</v>
+      </c>
+      <c r="M88" s="7">
+        <v>0</v>
+      </c>
+      <c r="N88" s="7"/>
+      <c r="O88" s="7">
+        <v>501555</v>
+      </c>
+      <c r="P88" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q88" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="R88" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S88" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="89" spans="1:19" ht="46" x14ac:dyDescent="0.2">
+      <c r="A89" s="2">
+        <v>10</v>
+      </c>
+      <c r="B89" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C89" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D89" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="E89" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="F89" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="G89" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="H89" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I89" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J89" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="K89" s="7">
+        <v>530000</v>
+      </c>
+      <c r="L89" s="7">
+        <v>0</v>
+      </c>
+      <c r="M89" s="7">
+        <v>0</v>
+      </c>
+      <c r="N89" s="7"/>
+      <c r="O89" s="7">
+        <v>530000</v>
+      </c>
+      <c r="P89" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q89" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="R89" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S89" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="90" spans="1:19" ht="46" x14ac:dyDescent="0.2">
+      <c r="A90" s="2">
+        <v>11</v>
+      </c>
+      <c r="B90" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C90" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D90" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="E90" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="F90" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="G90" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="H90" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I90" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J90" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="K90" s="7">
+        <v>350000</v>
+      </c>
+      <c r="L90" s="7">
+        <v>0</v>
+      </c>
+      <c r="M90" s="7">
+        <v>0</v>
+      </c>
+      <c r="N90" s="7"/>
+      <c r="O90" s="7">
+        <v>350000</v>
+      </c>
+      <c r="P90" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q90" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="R90" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S90" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="91" spans="1:19" ht="46" x14ac:dyDescent="0.2">
+      <c r="A91" s="2">
+        <v>12</v>
+      </c>
+      <c r="B91" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C91" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D91" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="E91" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="F91" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="G91" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="H91" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I91" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J91" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="K91" s="7">
+        <v>350000</v>
+      </c>
+      <c r="L91" s="7">
+        <v>0</v>
+      </c>
+      <c r="M91" s="7">
+        <v>0</v>
+      </c>
+      <c r="N91" s="7"/>
+      <c r="O91" s="7">
+        <v>350000</v>
+      </c>
+      <c r="P91" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q91" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="R91" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S91" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="92" spans="1:19" ht="46" x14ac:dyDescent="0.2">
+      <c r="A92" s="2">
+        <v>13</v>
+      </c>
+      <c r="B92" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C92" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D92" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="E92" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="F92" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="G92" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="H92" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I92" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J92" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="K92" s="7">
+        <v>550000</v>
+      </c>
+      <c r="L92" s="7">
+        <v>0</v>
+      </c>
+      <c r="M92" s="7">
+        <v>0</v>
+      </c>
+      <c r="N92" s="7"/>
+      <c r="O92" s="7">
+        <v>550000</v>
+      </c>
+      <c r="P92" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q92" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="R92" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S92" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="93" spans="1:19" ht="46" x14ac:dyDescent="0.2">
+      <c r="A93" s="2">
+        <v>14</v>
+      </c>
+      <c r="B93" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C93" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D93" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="E93" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="F93" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="G93" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="H93" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I93" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J93" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="K93" s="7">
+        <v>397680</v>
+      </c>
+      <c r="L93" s="7">
+        <v>0</v>
+      </c>
+      <c r="M93" s="7">
+        <v>0</v>
+      </c>
+      <c r="N93" s="7"/>
+      <c r="O93" s="7">
+        <v>397680</v>
+      </c>
+      <c r="P93" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q93" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="R93" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S93" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="94" spans="1:19" ht="46" x14ac:dyDescent="0.2">
+      <c r="A94" s="2">
+        <v>15</v>
+      </c>
+      <c r="B94" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C94" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D94" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="E94" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="F94" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="G94" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="H94" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I94" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J94" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="K94" s="7">
+        <v>400000</v>
+      </c>
+      <c r="L94" s="7">
+        <v>0</v>
+      </c>
+      <c r="M94" s="7">
+        <v>0</v>
+      </c>
+      <c r="N94" s="7"/>
+      <c r="O94" s="7">
+        <v>400000</v>
+      </c>
+      <c r="P94" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q94" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="R94" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S94" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="95" spans="1:19" ht="46" x14ac:dyDescent="0.2">
+      <c r="A95" s="2">
+        <v>16</v>
+      </c>
+      <c r="B95" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C95" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D95" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="E95" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="F95" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="G95" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="H95" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I95" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J95" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="K95" s="7">
+        <v>500000</v>
+      </c>
+      <c r="L95" s="7">
+        <v>0</v>
+      </c>
+      <c r="M95" s="7">
+        <v>0</v>
+      </c>
+      <c r="N95" s="7"/>
+      <c r="O95" s="7">
+        <v>500000</v>
+      </c>
+      <c r="P95" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q95" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="R95" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S95" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="96" spans="1:19" ht="46" x14ac:dyDescent="0.2">
+      <c r="A96" s="2">
+        <v>17</v>
+      </c>
+      <c r="B96" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C96" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D96" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="E96" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="F96" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="G96" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="H96" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I96" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J96" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="K96" s="7">
+        <v>550020</v>
+      </c>
+      <c r="L96" s="7">
+        <v>0</v>
+      </c>
+      <c r="M96" s="7">
+        <v>0</v>
+      </c>
+      <c r="N96" s="7"/>
+      <c r="O96" s="7">
+        <v>550020</v>
+      </c>
+      <c r="P96" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q96" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="R96" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S96" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="97" spans="1:19" ht="46" x14ac:dyDescent="0.2">
+      <c r="A97" s="2">
+        <v>18</v>
+      </c>
+      <c r="B97" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C97" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D97" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="E97" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="F97" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="G97" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="H97" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I97" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J97" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="K97" s="7">
+        <v>581585</v>
+      </c>
+      <c r="L97" s="7">
+        <v>0</v>
+      </c>
+      <c r="M97" s="7">
+        <v>0</v>
+      </c>
+      <c r="N97" s="7"/>
+      <c r="O97" s="7">
+        <v>581585</v>
+      </c>
+      <c r="P97" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q97" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="R97" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S97" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="98" spans="1:19" ht="46" x14ac:dyDescent="0.2">
+      <c r="A98" s="2">
+        <v>19</v>
+      </c>
+      <c r="B98" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C98" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D98" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="E98" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="F98" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="G98" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="H98" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I98" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J98" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="K98" s="7">
+        <v>290000</v>
+      </c>
+      <c r="L98" s="7">
+        <v>0</v>
+      </c>
+      <c r="M98" s="7">
+        <v>0</v>
+      </c>
+      <c r="N98" s="7"/>
+      <c r="O98" s="7">
+        <v>290000</v>
+      </c>
+      <c r="P98" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q98" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="R98" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S98" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="99" spans="1:19" ht="46" x14ac:dyDescent="0.2">
+      <c r="A99" s="2">
+        <v>20</v>
+      </c>
+      <c r="B99" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C99" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D99" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="E99" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="F99" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="G99" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="H99" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I99" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J99" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="K99" s="7">
+        <v>550000</v>
+      </c>
+      <c r="L99" s="7">
+        <v>0</v>
+      </c>
+      <c r="M99" s="7">
+        <v>0</v>
+      </c>
+      <c r="N99" s="7"/>
+      <c r="O99" s="7">
+        <v>550000</v>
+      </c>
+      <c r="P99" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q99" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="R99" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S99" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="100" spans="1:19" ht="46" x14ac:dyDescent="0.2">
+      <c r="A100" s="2">
+        <v>21</v>
+      </c>
+      <c r="B100" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C100" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D100" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="E100" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="F100" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="G100" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="H100" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I100" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J100" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="K100" s="7">
+        <v>450000</v>
+      </c>
+      <c r="L100" s="7">
+        <v>0</v>
+      </c>
+      <c r="M100" s="7">
+        <v>0</v>
+      </c>
+      <c r="N100" s="7"/>
+      <c r="O100" s="7">
+        <v>450000</v>
+      </c>
+      <c r="P100" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q100" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="R100" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S100" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="101" spans="1:19" ht="46" x14ac:dyDescent="0.2">
+      <c r="A101" s="2">
+        <v>22</v>
+      </c>
+      <c r="B101" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C101" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D101" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="E101" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="F101" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="G101" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="H101" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I101" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J101" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="K101" s="7">
+        <v>500000</v>
+      </c>
+      <c r="L101" s="7">
+        <v>0</v>
+      </c>
+      <c r="M101" s="7">
+        <v>0</v>
+      </c>
+      <c r="N101" s="7"/>
+      <c r="O101" s="7">
+        <v>500000</v>
+      </c>
+      <c r="P101" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q101" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="R101" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S101" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="102" spans="1:19" ht="46" x14ac:dyDescent="0.2">
+      <c r="A102" s="2">
+        <v>23</v>
+      </c>
+      <c r="B102" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C102" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D102" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="E102" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="F102" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="G102" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="H102" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I102" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J102" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="K102" s="7">
+        <v>493000</v>
+      </c>
+      <c r="L102" s="7">
+        <v>0</v>
+      </c>
+      <c r="M102" s="7">
+        <v>0</v>
+      </c>
+      <c r="N102" s="7"/>
+      <c r="O102" s="7">
+        <v>493000</v>
+      </c>
+      <c r="P102" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q102" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="R102" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S102" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="103" spans="1:19" ht="61" x14ac:dyDescent="0.2">
+      <c r="A103" s="2">
+        <v>24</v>
+      </c>
+      <c r="B103" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C103" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="D103" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="E103" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="F103" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="G103" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="H103" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I103" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J103" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="K103" s="7">
+        <v>152092594</v>
+      </c>
+      <c r="L103" s="7">
+        <v>12167406</v>
+      </c>
+      <c r="M103" s="7">
+        <v>0</v>
+      </c>
+      <c r="N103" s="7"/>
+      <c r="O103" s="7">
+        <v>164260000</v>
+      </c>
+      <c r="P103" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q103" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="R103" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S103" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="104" spans="1:19" ht="46" x14ac:dyDescent="0.2">
+      <c r="A104" s="2">
+        <v>25</v>
+      </c>
+      <c r="B104" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C104" s="6" t="s">
+        <v>270</v>
+      </c>
+      <c r="D104" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="E104" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="F104" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="G104" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="H104" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I104" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J104" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="K104" s="7">
+        <v>4946000</v>
+      </c>
+      <c r="L104" s="7">
+        <v>395680</v>
+      </c>
+      <c r="M104" s="7"/>
+      <c r="N104" s="7"/>
+      <c r="O104" s="7">
+        <v>5341680</v>
+      </c>
+      <c r="P104" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q104" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="R104" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S104" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="105" spans="1:19" ht="46" x14ac:dyDescent="0.2">
+      <c r="A105" s="2">
+        <v>26</v>
+      </c>
+      <c r="B105" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C105" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="D105" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="E105" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="F105" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="G105" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="H105" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I105" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="J105" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="K105" s="7">
+        <v>834280</v>
+      </c>
+      <c r="L105" s="7">
+        <v>66742</v>
+      </c>
+      <c r="M105" s="7"/>
+      <c r="N105" s="7"/>
+      <c r="O105" s="7">
+        <v>901022</v>
+      </c>
+      <c r="P105" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q105" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="R105" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S105" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="106" spans="1:19" ht="31" x14ac:dyDescent="0.2">
+      <c r="A106" s="2">
+        <v>27</v>
+      </c>
+      <c r="B106" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C106" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="D106" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="E106" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="F106" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="G106" s="6" t="s">
+        <v>279</v>
+      </c>
+      <c r="H106" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I106" s="6" t="s">
+        <v>280</v>
+      </c>
+      <c r="J106" s="6" t="s">
+        <v>281</v>
+      </c>
+      <c r="K106" s="7">
+        <v>909091</v>
+      </c>
+      <c r="L106" s="7">
+        <v>90909</v>
+      </c>
+      <c r="M106" s="7"/>
+      <c r="N106" s="7"/>
+      <c r="O106" s="7">
+        <v>1000000</v>
+      </c>
+      <c r="P106" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q106" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="R106" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S106" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="107" spans="1:19" ht="31" x14ac:dyDescent="0.2">
+      <c r="A107" s="2">
+        <v>28</v>
+      </c>
+      <c r="B107" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C107" s="6" t="s">
+        <v>282</v>
+      </c>
+      <c r="D107" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="E107" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="F107" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="G107" s="6" t="s">
+        <v>286</v>
+      </c>
+      <c r="H107" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I107" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J107" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="K107" s="7">
+        <v>17300000</v>
+      </c>
+      <c r="L107" s="7">
+        <v>1384000</v>
+      </c>
+      <c r="M107" s="7">
+        <v>0</v>
+      </c>
+      <c r="N107" s="7"/>
+      <c r="O107" s="7">
+        <v>18684000</v>
+      </c>
+      <c r="P107" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q107" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="R107" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S107" s="6" t="s">
         <v>33</v>
       </c>
     </row>

</xml_diff>